<commit_message>
MO-430 - renistate locales + translations - fixes en & cy locales JSON - regenerate translations
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/00-shared-layout.xlsx
+++ b/translations/welsh-translations/xlsx/00-shared-layout.xlsx
@@ -271,6 +271,15 @@
     <t>Rheoli’r cyfrif</t>
   </si>
   <si>
+    <t>common.nav.signIn</t>
+  </si>
+  <si>
+    <t>Sign in</t>
+  </si>
+  <si>
+    <t>Mewngofnodi</t>
+  </si>
+  <si>
     <t>common.nav.signOut</t>
   </si>
   <si>
@@ -278,15 +287,6 @@
   </si>
   <si>
     <t>Allgofnodi</t>
-  </si>
-  <si>
-    <t>common.nav.signIn</t>
-  </si>
-  <si>
-    <t>Sign in</t>
-  </si>
-  <si>
-    <t>Mewngofnodi</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
add new manage obligations page
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/00-shared-layout.xlsx
+++ b/translations/welsh-translations/xlsx/00-shared-layout.xlsx
@@ -1,21 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8EAE257-5DF8-4F82-9548-1AFA6AD97DAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Welsh translations" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Welsh translations" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="92">
   <si>
     <t>Translator notes</t>
   </si>
@@ -38,6 +34,9 @@
     <t>Welsh</t>
   </si>
   <si>
+    <t>Figma link</t>
+  </si>
+  <si>
     <t>common.serviceName</t>
   </si>
   <si>
@@ -50,6 +49,9 @@
     <t>Report packaging data</t>
   </si>
   <si>
+    <t>Riportio data pecynwaith</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
@@ -68,6 +70,9 @@
     <t>Show or hide menu</t>
   </si>
   <si>
+    <t>Dangos neu guddio'r ddewislen</t>
+  </si>
+  <si>
     <t>common.phaseBanner.lead</t>
   </si>
   <si>
@@ -107,15 +112,24 @@
     <t>Beta banner</t>
   </si>
   <si>
+    <t>Baner beta</t>
+  </si>
+  <si>
     <t>common.languageSwitcher.label</t>
   </si>
   <si>
     <t>Language</t>
   </si>
   <si>
+    <t>Iaith</t>
+  </si>
+  <si>
     <t>common.languageSwitcher.english</t>
   </si>
   <si>
+    <t>Saesneg</t>
+  </si>
+  <si>
     <t>common.languageSwitcher.welsh</t>
   </si>
   <si>
@@ -146,6 +160,9 @@
     <t>Email</t>
   </si>
   <si>
+    <t>E-bost</t>
+  </si>
+  <si>
     <t>common.footer.telephone</t>
   </si>
   <si>
@@ -251,6 +268,18 @@
     <t>Manage account</t>
   </si>
   <si>
+    <t>Rheoli’r cyfrif</t>
+  </si>
+  <si>
+    <t>common.nav.signOut</t>
+  </si>
+  <si>
+    <t>Sign out</t>
+  </si>
+  <si>
+    <t>Allgofnodi</t>
+  </si>
+  <si>
     <t>common.nav.signIn</t>
   </si>
   <si>
@@ -258,68 +287,27 @@
   </si>
   <si>
     <t>Mewngofnodi</t>
-  </si>
-  <si>
-    <t>common.nav.signOut</t>
-  </si>
-  <si>
-    <t>Sign out</t>
-  </si>
-  <si>
-    <t>Allgofnodi</t>
-  </si>
-  <si>
-    <t>Figma link for this content</t>
-  </si>
-  <si>
-    <t>There is no Figma link for this content.</t>
-  </si>
-  <si>
-    <t>Riportio data pecynwaith</t>
-  </si>
-  <si>
-    <t>Dangos neu guddio'r ddewislen</t>
-  </si>
-  <si>
-    <t>Baner beta</t>
-  </si>
-  <si>
-    <t>Iaith</t>
-  </si>
-  <si>
-    <t>Saesneg</t>
-  </si>
-  <si>
-    <t>E-bost</t>
-  </si>
-  <si>
-    <t>Rheoli’r cyfrif</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -347,18 +335,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -699,9 +684,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F32"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
     <col min="2" max="3" width="35" hidden="1" customWidth="1"/>
@@ -709,608 +694,608 @@
     <col min="6" max="6" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D1" s="3" t="s">
+    <row r="1" ht="24" customHeight="1" spans="4:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-    </row>
-    <row r="2" spans="1:6" s="1" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D2" s="4" t="s">
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" ht="36" customHeight="1" spans="4:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-    </row>
-    <row r="3" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:6" s="2" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" ht="36" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="24" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F4" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>86</v>
+        <v>12</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>87</v>
+        <v>19</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>89</v>
+        <v>36</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="F14" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E18" s="1" t="s">
+      <c r="E32" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>83</v>
-      </c>
       <c r="F32" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F32" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A4:F32"/>
   <mergeCells count="2">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
MO-515/516: add GA analytics and update cookie page
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/00-shared-layout.xlsx
+++ b/translations/welsh-translations/xlsx/00-shared-layout.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="125">
   <si>
     <t>Translator notes</t>
   </si>
@@ -37,22 +37,121 @@
     <t>Figma link</t>
   </si>
   <si>
+    <t>cookies.banner.essentialParagraph</t>
+  </si>
+  <si>
+    <t>shared-layout</t>
+  </si>
+  <si>
+    <t>Shared layout, header, navigation, language switcher and footer</t>
+  </si>
+  <si>
+    <t>We use some essential cookies to make this service work.</t>
+  </si>
+  <si>
+    <t>Rydyn ni’n defnyddio cwcis hanfodol i wneud i’r gwasanaeth yma weithio.</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>cookies.banner.analyticsParagraph</t>
+  </si>
+  <si>
+    <t>We’d also like to use analytics cookies so we can understand how you use the service and make improvements.</t>
+  </si>
+  <si>
+    <t>Hoffen ni hefyd ddefnyddio cwcis dadansoddeg er mwyn deall sut rydych chi’n defnyddio’r gwasanaeth a gwneud gwelliannau.</t>
+  </si>
+  <si>
+    <t>cookies.banner.accepted</t>
+  </si>
+  <si>
+    <t>You’ve accepted analytics cookies. You can</t>
+  </si>
+  <si>
+    <t>Rydych chi wedi derbyn cwcis dadansoddeg. Gallwch chi</t>
+  </si>
+  <si>
+    <t>cookies.banner.changeSettings</t>
+  </si>
+  <si>
+    <t>change your cookie settings</t>
+  </si>
+  <si>
+    <t>newid eich gosodiadau cwcis</t>
+  </si>
+  <si>
+    <t>cookies.banner.atAnyTime</t>
+  </si>
+  <si>
+    <t>at any time.</t>
+  </si>
+  <si>
+    <t>unrhyw bryd.</t>
+  </si>
+  <si>
+    <t>cookies.banner.rejected</t>
+  </si>
+  <si>
+    <t>You’ve rejected analytics cookies. You can</t>
+  </si>
+  <si>
+    <t>Rydych chi wedi gwrthod cwcis dadansoddeg. Gallwch chi</t>
+  </si>
+  <si>
+    <t>cookies.banner.title</t>
+  </si>
+  <si>
+    <t>Cookies on the ‘report packaging data’ service</t>
+  </si>
+  <si>
+    <t>Cwcis ar y gwasanaeth ‘Rhoi gwybod am ddata pecynwaith’</t>
+  </si>
+  <si>
+    <t>cookies.banner.accept</t>
+  </si>
+  <si>
+    <t>Accept analytics cookies</t>
+  </si>
+  <si>
+    <t>Derbyn cwcis dadansoddeg</t>
+  </si>
+  <si>
+    <t>cookies.banner.reject</t>
+  </si>
+  <si>
+    <t>Reject analytics cookies</t>
+  </si>
+  <si>
+    <t>Gwrthod cwcis dadansoddeg</t>
+  </si>
+  <si>
+    <t>cookies.banner.viewCookies</t>
+  </si>
+  <si>
+    <t>View cookies</t>
+  </si>
+  <si>
+    <t>Gweld cwcis</t>
+  </si>
+  <si>
+    <t>cookies.banner.hide</t>
+  </si>
+  <si>
+    <t>Hide cookie message</t>
+  </si>
+  <si>
+    <t>Cuddio’r neges ynghylch cwcis</t>
+  </si>
+  <si>
     <t>common.serviceName</t>
   </si>
   <si>
-    <t>shared-layout</t>
-  </si>
-  <si>
-    <t>Shared layout, header, navigation, language switcher and footer</t>
-  </si>
-  <si>
     <t>Report packaging data</t>
   </si>
   <si>
     <t>Riportio data pecynwaith</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>common.nav.menu</t>
@@ -685,7 +784,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -749,7 +848,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -863,7 +962,7 @@
         <v>30</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>13</v>
@@ -871,7 +970,7 @@
     </row>
     <row r="12" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>9</v>
@@ -880,10 +979,10 @@
         <v>10</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>13</v>
@@ -891,7 +990,7 @@
     </row>
     <row r="13" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>9</v>
@@ -900,10 +999,10 @@
         <v>10</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>13</v>
@@ -911,7 +1010,7 @@
     </row>
     <row r="14" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>9</v>
@@ -920,10 +1019,10 @@
         <v>10</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>13</v>
@@ -931,7 +1030,7 @@
     </row>
     <row r="15" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>9</v>
@@ -940,10 +1039,10 @@
         <v>10</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>13</v>
@@ -951,7 +1050,7 @@
     </row>
     <row r="16" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>9</v>
@@ -960,10 +1059,10 @@
         <v>10</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>13</v>
@@ -971,7 +1070,7 @@
     </row>
     <row r="17" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>9</v>
@@ -980,10 +1079,10 @@
         <v>10</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>13</v>
@@ -991,7 +1090,7 @@
     </row>
     <row r="18" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>9</v>
@@ -1000,10 +1099,10 @@
         <v>10</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>13</v>
@@ -1011,7 +1110,7 @@
     </row>
     <row r="19" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>9</v>
@@ -1020,10 +1119,10 @@
         <v>10</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>13</v>
@@ -1031,7 +1130,7 @@
     </row>
     <row r="20" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>9</v>
@@ -1040,10 +1139,10 @@
         <v>10</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>13</v>
@@ -1051,7 +1150,7 @@
     </row>
     <row r="21" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>9</v>
@@ -1060,10 +1159,10 @@
         <v>10</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>13</v>
@@ -1071,7 +1170,7 @@
     </row>
     <row r="22" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>9</v>
@@ -1080,10 +1179,10 @@
         <v>10</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>61</v>
+        <v>13</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>13</v>
@@ -1091,7 +1190,7 @@
     </row>
     <row r="23" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>9</v>
@@ -1100,10 +1199,10 @@
         <v>10</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>13</v>
@@ -1111,7 +1210,7 @@
     </row>
     <row r="24" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>9</v>
@@ -1120,10 +1219,10 @@
         <v>10</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>13</v>
@@ -1131,7 +1230,7 @@
     </row>
     <row r="25" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>9</v>
@@ -1140,10 +1239,10 @@
         <v>10</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>69</v>
+        <v>5</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>13</v>
@@ -1151,7 +1250,7 @@
     </row>
     <row r="26" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>9</v>
@@ -1160,10 +1259,10 @@
         <v>10</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>73</v>
+        <v>13</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>13</v>
@@ -1289,8 +1388,228 @@
         <v>13</v>
       </c>
     </row>
+    <row r="33" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:F32"/>
+  <autoFilter ref="A4:F43"/>
   <mergeCells count="2">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>

</xml_diff>

<commit_message>
use GA & GTM env as feature flag
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/00-shared-layout.xlsx
+++ b/translations/welsh-translations/xlsx/00-shared-layout.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="128">
   <si>
     <t>Translator notes</t>
   </si>
@@ -37,24 +37,33 @@
     <t>Figma link</t>
   </si>
   <si>
+    <t>cookies.banner.title</t>
+  </si>
+  <si>
+    <t>shared-layout</t>
+  </si>
+  <si>
+    <t>Shared layout, header, navigation, language switcher and footer</t>
+  </si>
+  <si>
+    <t>Cookies on the ‘report packaging data’ service</t>
+  </si>
+  <si>
+    <t>Cwcis ar y gwasanaeth ‘Rhoi gwybod am ddata pecynwaith’</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>cookies.banner.essentialParagraph</t>
   </si>
   <si>
-    <t>shared-layout</t>
-  </si>
-  <si>
-    <t>Shared layout, header, navigation, language switcher and footer</t>
-  </si>
-  <si>
     <t>We use some essential cookies to make this service work.</t>
   </si>
   <si>
     <t>Rydyn ni’n defnyddio cwcis hanfodol i wneud i’r gwasanaeth yma weithio.</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>cookies.banner.analyticsParagraph</t>
   </si>
   <si>
@@ -100,15 +109,6 @@
     <t>Rydych chi wedi gwrthod cwcis dadansoddeg. Gallwch chi</t>
   </si>
   <si>
-    <t>cookies.banner.title</t>
-  </si>
-  <si>
-    <t>Cookies on the ‘report packaging data’ service</t>
-  </si>
-  <si>
-    <t>Cwcis ar y gwasanaeth ‘Rhoi gwybod am ddata pecynwaith’</t>
-  </si>
-  <si>
     <t>cookies.banner.accept</t>
   </si>
   <si>
@@ -143,6 +143,15 @@
   </si>
   <si>
     <t>Cuddio’r neges ynghylch cwcis</t>
+  </si>
+  <si>
+    <t>common.nav.skipToMainContent</t>
+  </si>
+  <si>
+    <t>Skip to main content</t>
+  </si>
+  <si>
+    <t>Neidio i’r prif gynnwys</t>
   </si>
   <si>
     <t>common.serviceName</t>
@@ -784,7 +793,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -848,7 +857,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -868,7 +877,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
@@ -1182,7 +1191,7 @@
         <v>63</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>13</v>
@@ -1190,7 +1199,7 @@
     </row>
     <row r="23" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>9</v>
@@ -1199,10 +1208,10 @@
         <v>10</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>66</v>
+        <v>13</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>13</v>
@@ -1239,10 +1248,10 @@
         <v>10</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>5</v>
+        <v>71</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>13</v>
@@ -1250,7 +1259,7 @@
     </row>
     <row r="26" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>9</v>
@@ -1259,10 +1268,10 @@
         <v>10</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>73</v>
+        <v>5</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>13</v>
+        <v>74</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>13</v>
@@ -1270,7 +1279,7 @@
     </row>
     <row r="27" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>9</v>
@@ -1279,10 +1288,10 @@
         <v>10</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>76</v>
+        <v>13</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>13</v>
@@ -1608,8 +1617,28 @@
         <v>13</v>
       </c>
     </row>
+    <row r="44" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:F43"/>
+  <autoFilter ref="A4:F44"/>
   <mergeCells count="2">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>

</xml_diff>